<commit_message>
Checkpoint docs 19/20/21 enrichment + BPS interface spec; ignore credentialed notebooks
- Add end-to-end walkthrough (doc 20) and field-level lineage (doc 21), zh+en
- Expand doc 14 BPS-driven servicer FCL interface; enrich doc 19 sample dump
  with per-table business meaning + full upstream/downstream lineage
- Update docs 02/05/06/07/13, data dictionary, fcl_pipeline.html
- Track single-source outputs (fcl_table_meta.json, verify/consol JSON,
  sample dump data) + new generator scripts
- gitignore *.ipynb / *.pdf / editor "- Copy" files: download notebooks held
  hardcoded AWS keys (never committed; keys should be rotated)
- CLAUDE.md: add Python-exec (endpoint-security) inline-execution rule

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/16_bps_fcl_display_mapping.xlsx
+++ b/docs/16_bps_fcl_display_mapping.xlsx
@@ -279,6 +279,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -309,6 +312,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -339,6 +345,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -369,6 +378,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -399,6 +411,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -429,6 +444,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -459,6 +477,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -1083,7 +1104,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A43:F110"/>
+  <dimension ref="A1:F110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -1094,6 +1115,48 @@
     <col width="26" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
+    <row r="1"/>
+    <row r="2"/>
+    <row r="3"/>
+    <row r="4"/>
+    <row r="5"/>
+    <row r="6"/>
+    <row r="7"/>
+    <row r="8"/>
+    <row r="9"/>
+    <row r="10"/>
+    <row r="11"/>
+    <row r="12"/>
+    <row r="13"/>
+    <row r="14"/>
+    <row r="15"/>
+    <row r="16"/>
+    <row r="17"/>
+    <row r="18"/>
+    <row r="19"/>
+    <row r="20"/>
+    <row r="21"/>
+    <row r="22"/>
+    <row r="23"/>
+    <row r="24"/>
+    <row r="25"/>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
+    <row r="40"/>
+    <row r="41"/>
+    <row r="42"/>
     <row r="43" ht="22" customHeight="1">
       <c r="A43" s="1" t="inlineStr">
         <is>
@@ -1173,6 +1236,8 @@
         </is>
       </c>
     </row>
+    <row r="50"/>
+    <row r="51"/>
     <row r="52" ht="22" customHeight="1">
       <c r="A52" s="1" t="inlineStr">
         <is>
@@ -1396,7 +1461,7 @@
       </c>
       <c r="D62" s="5" t="inlineStr">
         <is>
-          <t>如果 currentmilestone 非空，则 summary_current_step = currentmilestone；否则 = fcstage</t>
+          <t>如果 currentmilestone 非空，则 summary_current_step = currentmilestone；否则 = fcstage　⚠️ 实测存疑（doc 19，2026-06-04）：BPS 实际取 fcstage，currentmilestone 非空仍未用——取值顺序待 ETL 代码核实，见 doc 13 Q13</t>
         </is>
       </c>
     </row>
@@ -1462,7 +1527,7 @@
       </c>
       <c r="D65" s="6" t="inlineStr">
         <is>
-          <t>直接取值</t>
+          <t>直接取值　⚠️ 实测未填充（doc 19，2026-06-04）：Newrez 源有值但 BPS 该列为空（同源 summary_firm / timeline_referred_to_foreclosure 却有值＝部分填充），见 doc 13 Q14</t>
         </is>
       </c>
     </row>
@@ -1484,7 +1549,7 @@
       </c>
       <c r="D66" s="5" t="inlineStr">
         <is>
-          <t>如果 activefcflag=0，则 summary_completed_foreclosure = 1；如果 activefcflag=1，则 = 0（即对 activefcflag 取反）。⚠️ activefcflag=0 = 当前不处于活跃止赎流程（含撤销/复议/付清/完成），并非都已完成</t>
+          <t>如果 activefcflag=0，则 summary_completed_foreclosure = 1；如果 activefcflag=1，则 = 0（即对 activefcflag 取反）。⚠️ activefcflag=0 = 当前不处于活跃止赎流程（含撤销/复议/付清/完成），并非都已完成　⚠️ 实测未填充（doc 19，2026-06-04）：Newrez 源有值但 BPS 该列为空（同源 summary_firm / timeline_referred_to_foreclosure 却有值＝部分填充），见 doc 13 Q14</t>
         </is>
       </c>
     </row>
@@ -1550,10 +1615,11 @@
       </c>
       <c r="D69" s="6" t="inlineStr">
         <is>
-          <t>直接取值</t>
-        </is>
-      </c>
-    </row>
+          <t>直接取值　⚠️ 实测未填充（doc 19，2026-06-04）：Newrez 源有值但 BPS 该列为空（同源 summary_firm / timeline_referred_to_foreclosure 却有值＝部分填充），见 doc 13 Q14</t>
+        </is>
+      </c>
+    </row>
+    <row r="70"/>
     <row r="71">
       <c r="A71" s="8" t="inlineStr">
         <is>
@@ -2144,6 +2210,7 @@
         </is>
       </c>
     </row>
+    <row r="91"/>
     <row r="92" ht="22" customHeight="1">
       <c r="A92" s="1" t="inlineStr">
         <is>
@@ -2663,6 +2730,7 @@
         </is>
       </c>
     </row>
+    <row r="109"/>
     <row r="110">
       <c r="A110" s="8" t="inlineStr">
         <is>
@@ -2690,7 +2758,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A47:F118"/>
+  <dimension ref="A1:F118"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -2701,6 +2769,52 @@
     <col width="26" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
+    <row r="1"/>
+    <row r="2"/>
+    <row r="3"/>
+    <row r="4"/>
+    <row r="5"/>
+    <row r="6"/>
+    <row r="7"/>
+    <row r="8"/>
+    <row r="9"/>
+    <row r="10"/>
+    <row r="11"/>
+    <row r="12"/>
+    <row r="13"/>
+    <row r="14"/>
+    <row r="15"/>
+    <row r="16"/>
+    <row r="17"/>
+    <row r="18"/>
+    <row r="19"/>
+    <row r="20"/>
+    <row r="21"/>
+    <row r="22"/>
+    <row r="23"/>
+    <row r="24"/>
+    <row r="25"/>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
+    <row r="40"/>
+    <row r="41"/>
+    <row r="42"/>
+    <row r="43"/>
+    <row r="44"/>
+    <row r="45"/>
+    <row r="46"/>
     <row r="47" ht="22" customHeight="1">
       <c r="A47" s="1" t="inlineStr">
         <is>
@@ -2780,6 +2894,8 @@
         </is>
       </c>
     </row>
+    <row r="54"/>
+    <row r="55"/>
     <row r="56" ht="22" customHeight="1">
       <c r="A56" s="1" t="inlineStr">
         <is>
@@ -2827,7 +2943,7 @@
       </c>
       <c r="D58" s="5" t="inlineStr">
         <is>
-          <t>直接取值</t>
+          <t>直接取值　⚠️ 实测未填充（doc 19，2026-06-04）：Newrez 源有值但 BPS 该列为空（同源 summary_firm / timeline_referred_to_foreclosure 却有值＝部分填充），见 doc 13 Q14</t>
         </is>
       </c>
     </row>
@@ -2849,7 +2965,7 @@
       </c>
       <c r="D59" s="6" t="inlineStr">
         <is>
-          <t>直接取值</t>
+          <t>直接取值　⚠️ 实测未填充（doc 19，2026-06-04）：Newrez 源有值但 BPS 该列为空（同源 summary_firm / timeline_referred_to_foreclosure 却有值＝部分填充），见 doc 13 Q14</t>
         </is>
       </c>
     </row>
@@ -2871,7 +2987,7 @@
       </c>
       <c r="D60" s="5" t="inlineStr">
         <is>
-          <t>直接取值</t>
+          <t>直接取值　⚠️ 实测未填充（doc 19，2026-06-04）：Newrez 源有值但 BPS 该列为空（同源 summary_firm / timeline_referred_to_foreclosure 却有值＝部分填充），见 doc 13 Q14</t>
         </is>
       </c>
     </row>
@@ -2893,7 +3009,7 @@
       </c>
       <c r="D61" s="6" t="inlineStr">
         <is>
-          <t>直接取值</t>
+          <t>直接取值　⚠️ 实测未填充（doc 19，2026-06-04）：Newrez 源有值但 BPS 该列为空（同源 summary_firm / timeline_referred_to_foreclosure 却有值＝部分填充），见 doc 13 Q14</t>
         </is>
       </c>
     </row>
@@ -3179,7 +3295,7 @@
       </c>
       <c r="D74" s="5" t="inlineStr">
         <is>
-          <t>COALESCE(dtdeedrecorded, fcremovaldate)</t>
+          <t>COALESCE(dtdeedrecorded, fcremovaldate)　⚠️ 实测未填充（doc 19，2026-06-04）：Newrez 源有值但 BPS 该列为空（同源 summary_firm / timeline_referred_to_foreclosure 却有值＝部分填充），见 doc 13 Q14</t>
         </is>
       </c>
     </row>
@@ -3227,6 +3343,7 @@
         </is>
       </c>
     </row>
+    <row r="77"/>
     <row r="78">
       <c r="A78" s="8" t="inlineStr">
         <is>
@@ -3721,6 +3838,7 @@
         </is>
       </c>
     </row>
+    <row r="95"/>
     <row r="96" ht="22" customHeight="1">
       <c r="A96" s="1" t="inlineStr">
         <is>
@@ -4368,6 +4486,7 @@
         </is>
       </c>
     </row>
+    <row r="117"/>
     <row r="118">
       <c r="A118" s="8" t="inlineStr">
         <is>
@@ -6588,8 +6707,8 @@
     <mergeCell ref="A54:F54"/>
     <mergeCell ref="A71:F71"/>
     <mergeCell ref="A52:F52"/>
+    <mergeCell ref="A85:F85"/>
     <mergeCell ref="A47:F47"/>
-    <mergeCell ref="A85:F85"/>
     <mergeCell ref="A66:F66"/>
     <mergeCell ref="A80:F80"/>
     <mergeCell ref="A34:F34"/>

</xml_diff>